<commit_message>
Regenerate the coverage workbook with NCLT, Bombay HC and IGR now wired in
Adds NCLT Case Status and Bombay High Court Case Status as confirmed-live
CIN-sheet findings, and updates the IGR Maharashtra registered-deed row to
note it is wired into run_igr_registered_deed_check -- moving it out of the
unmapped/unused sheet, since all three are now called from
run_company_charter rather than sitting unwired.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/RERA_Data_Coverage.xlsx
+++ b/docs/RERA_Data_Coverage.xlsx
@@ -16,8 +16,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'A - RERA by authority'!$A$4:$M$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'B - CTS land records'!$A$4:$F$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'C - CIN corporate'!$A$4:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'D - Available but unused'!$A$4:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'C - CIN corporate'!$A$4:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'D - Available but unused'!$A$4:$E$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,14 +52,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <strike val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -116,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -145,18 +137,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Regenerated 2026-08-31 by build_data_coverage.py</t>
+          <t>Regenerated 2026-09-23 by build_data_coverage.py</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2510,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Audited live 2026-09-01 with a REAL result, not just a reachable form. Two search modes, both free and CAPTCHA-gated (confirmed via DOM inspection, not just a page-text guess): 'Property Details' (Year -&gt; District -&gt; Village/Area, an autocomplete text field paired with a dropdown -&gt; Survey/CTS/Milkat/Gat/Plot No.; a name-based search is also offered once a property number is entered) and 'Document Number' (Registration Type [eFiling/eRegistration/Regular/iSarita 2.0] -&gt; District, all 37 -- this mode is genuinely statewide, not Mumbai-only -&gt; SRO -&gt; Year -&gt; Doc No.). Document Number/SRO Mumbai 9 (Andheri)/2024/#100 returned a real registered Leave &amp; License agreement dated 03/01/2024 -- Seller/Lessor 'Ramesh Babulal Shah', Purchaser/Lessee 'M/s Matushri Impex' (through partner Ramesh T. Bhalani), full property description (Bandra Kurla Complex premises, CTS No. 4207) AND consideration (monthly rent Rs 44,100 plus Rs 5,29,200 advance for the first 12 months) -- all present in the RESULT LIST ROW ITSELF, no further click needed. Each row also carries an 'IndexII' button (a further postback, __doPostBack('RegistrationGrid','indexII$0')) documented in the site's own User Guide as opening a fuller Index II view in a separate window -- present and clickable, but its own content was NOT captured this pass (the popup did not materialize in this environment), so that specific view stays unconfirmed rather than assumed. A real, stated limitation from the site's own FAQ: Power of Attorney and Will deeds are NOT available in search results. Mumbai city and Suburban districts go back to 1985; 'selected offices' elsewhere now reach back before the earlier 2002 baseline too, per the site's own notice.</t>
+          <t>Audited live 2026-09-01 with a REAL result, not just a reachable form. Two search modes, both free and CAPTCHA-gated (confirmed via DOM inspection, not just a page-text guess): 'Property Details' (Year -&gt; District -&gt; Village/Area, an autocomplete text field paired with a dropdown -&gt; Survey/CTS/Milkat/Gat/Plot No.; a name-based search is also offered once a property number is entered) and 'Document Number' (Registration Type [eFiling/eRegistration/Regular/iSarita 2.0] -&gt; District, all 37 -- this mode is genuinely statewide, not Mumbai-only -&gt; SRO -&gt; Year -&gt; Doc No.). Document Number/SRO Mumbai 9 (Andheri)/2024/#100 returned a real registered Leave &amp; License agreement dated 03/01/2024 -- Seller/Lessor 'Ramesh Babulal Shah', Purchaser/Lessee 'M/s Matushri Impex' (through partner Ramesh T. Bhalani), full property description (Bandra Kurla Complex premises, CTS No. 4207) AND consideration (monthly rent Rs 44,100 plus Rs 5,29,200 advance for the first 12 months) -- all present in the RESULT LIST ROW ITSELF, no further click needed. Each row also carries an 'IndexII' button (a further postback, __doPostBack('RegistrationGrid','indexII$0')) documented in the site's own User Guide as opening a fuller Index II view in a separate window -- present and clickable, but its own content was NOT captured this pass (the popup did not materialize in this environment), so that specific view stays unconfirmed rather than assumed. A real, stated limitation from the site's own FAQ: Power of Attorney and Will deeds are NOT available in search results. Mumbai city and Suburban districts go back to 1985; 'selected offices' elsewhere now reach back before the earlier 2002 baseline too, per the site's own notice. WIRED IN 2026-09-15 (run_igr_registered_deed_check): document-number search only, asked directly of a human at the terminal (district/SRO/year/doc-no, no candidate list) since a document number is either already in hand or not knowable at all; search_by_property() stays unwired since its result shape is still unconfirmed against a real row.</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3171,8 +3151,82 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>NCLT Case Status (direct tribunal query)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>NCLT e-filing Case Status portal, party-name search</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Free + CAPTCHA</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>confirmed-live</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>nclt_check</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>WIRED IN 2026-09-15. A DIRECT party-name query against the tribunal's own portal -- distinct from _safe_group_litigation's indirect Indian Kanoon name search just above. CAPTCHA-gated (one solve) and human-in-the-loop: only runs when a human is actually at this terminal, never headlessly. Mumbai Bench only; the other 15 benches nationwide are not searched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Bombay High Court Case Status (direct eCourts query)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Bombay HC eCourts Case Status, party-name search</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Free + CAPTCHA</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>confirmed-live</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>bombay_hc_check</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>WIRED IN 2026-09-15. A DIRECT party-name query, Original Side + Appellate Side (the two Bombay-city benches) across the last 5 registration years -- 10 separate CAPTCHA-gated lookups, since the portal requires a mandatory Registration Year per search. The other 5 benches (Aurangabad/Nagpur/Kolhapur/Goa/Special Court) are not searched by default. Used to also require an explicit human consent prompt before running, on top of the terminal check, given the 10x cost; removed 2026-09-23 once a human being present for every run of this pipeline was no longer in question.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G14"/>
+  <autoFilter ref="A4:G16"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -3187,7 +3241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3239,27 +3293,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Audited balance sheet / P&amp;L / ITR</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>GujRERA findoc</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Gujarat projects only</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Financial strength sub-metric currently scores None for every project. This would score it for GJ. RESOLVED 2026-08-28 for the single-project score (added to company_charter._HIGH_PRIORITY_DOC_KEYWORDS); the group-wide check (group_financial_disclosure.py) was widened 2026-09-09 to also cover West Bengal, Uttar Pradesh and Tamil Nadu -- though only Gujarat, Jharkhand, Haryana and West Bengal have a live-confirmed hit; UP and TN expose a searchable document list but have not produced one.</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Financial strength sub-metric currently scores None for every project. This would score it for GJ.</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3293,135 +3347,135 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>K-RERA defaulters list</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>K-RERA, observed</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Karnataka projects</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>No equivalent exists in any other authority. Direct red-flag input. RESOLVED 2026-09-09: adapter_karnataka.fetch_default_projects / search_default_projects_by_promoter reads K-RERA's own "Default Project List" (/viewDefaultProjects, 2,991 rows), wired into litigation_sweep.state_order_sweep via its new karnataka_defaults param.</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>No equivalent exists in any other authority. Direct red-flag input.</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>K-RERA projects under investigation</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>K-RERA, observed</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Karnataka projects</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Same -- a regulator-declared adverse signal. ALREADY COVERED, not a real gap: K-RERA's "Complaints under process" register (COMPLAINT_DETAILS_PAGE) has been part of _ORDER_REGISTERS / search_all_orders_by_promoter since the "Wire the seven unused registers" commit -- this finding predates that wiring and was stale.</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Same -- a regulator-declared adverse signal.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>K-RERA cost incurred vs estimated</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>K-RERA detail page</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Karnataka projects</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Financial-strength scores None everywhere today. This is a direct, free input. RESOLVED 2026-08-28 (per docs/PAN_INDIA_PROGRESS.md): cost incurred/estimated and extension history now render in company_charter._append_project_cost_extension_section, unconditional for K-RERA projects.</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Financial-strength scores None everywhere today. This is a direct, free input.</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>K-RERA delay reasons + NOC expiry</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>K-RERA detail page</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Karnataka projects</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Promoter-declared delay reasons and lapsed-NOC tracking; no equivalent elsewhere. RESOLVED 2026-09-09: adapter_karnataka._parse_detail now reads Delay Reason plus TWO distinct NOC tables (obtained-at-all status, and separately an obtained NOC's own expiry/renewal), rendered in company_charter._append_project_delay_noc_section. NOC "expiry tracking" specifically was empty on every project checked live -- the table is real, just rarely populated.</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Promoter-declared delay reasons and lapsed-NOC tracking; no equivalent elsewhere.</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Maha Bhulekh card fields</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Free portal, extraction broken</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Maharashtra projects</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Owner, area, tenure, encumbrance and mutation are all ON the card and none reach the document. RESOLVED 2026-08-24 (per docs/PAN_INDIA_PROGRESS.md): run_cts_land_lookup -&gt; company_charter._append_cts_land_record_section.</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Owner, area, tenure, encumbrance and mutation are all ON the card and none reach the document.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3430,22 +3484,22 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>IGR Maharashtra registered-deed search</t>
+          <t>JHARERA audited balance sheet + 3 years ITR</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>igr_maharashtra_search.py -- BUILT 2026-09-01, human-in-the-loop like up_captcha_search.py/cts_resolve.py, not wired into run_company_charter()</t>
+          <t>adapter_jharkhand.py document library (labelled, downloaded)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Maharashtra projects</t>
+          <t>Jharkhand projects</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>An independent, free, party-named check on registrations against a property/CTS number or a specific document number -- CAPTCHA-gated but otherwise unauthenticated. search_by_document_number() is confirmed against a real pulled result: seller/purchaser names, full property description and the ACTUAL CONSIDERATION AMOUNT in one row, no further click needed -- a direct corroboration (or contradiction) of a promoter's declared land dealings that nothing else in this pipeline checks independently. search_by_property() is also built and, confirmed live chasing a real Pune search, turned out to need THREE separate regions (mumbai/rest_of_maharashtra/urban), each its own field ids and cascade shape -- the landing page's default tab covers only the two Mumbai districts, not the whole state as it first appeared. A locality can sit in either the rural or urban region depending on how it was annexed: Pune's Market Yard (Gulatekadi) is under 'urban', not the rural taluka/village list a human would try first, and guessing wrong doesn't error -- it just returns a real but unrelated village list. All three regions' form mechanics are confirmed live end-to-end up to the CAPTCHA gate; the RESULT TABLE'S OWN SHAPE for search_by_property is still not confirmed against a real row for any of them, unlike document-number search. Also carries an integrated CERSAI cross-search on the same page, not yet driven by either function. A standalone script, run by a human, same as every other CAPTCHA-gated tool here -- not called from the automated Charter pipeline. DELIBERATELY NOT AUTOMATED, not a gap: CAPTCHA-gated and human-in-the-loop by design, same reasoning as cts_resolve.py/ts_rera_client.py -- wiring it into the unattended pipeline would need redesigning around the CAPTCHA, not just calling the existing script.</t>
+          <t>Same gap as GujRERA's findoc block: the financial-strength sub-metric scores None for every project regardless of state. This would score it for JH too.</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -3455,304 +3509,250 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>JHARERA audited balance sheet + 3 years ITR</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>adapter_jharkhand.py document library (labelled, downloaded)</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>JHARERA rejected + surrendered registration lists</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>REJECTED_LIST / SURRENDERED_LIST, imported into the adapter but never fetched</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Jharkhand projects</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Same gap as GujRERA's findoc block: the financial-strength sub-metric scores None for every project regardless of state. This would score it for JH too. RESOLVED 2026-08-28 for the single-project score (same fix as row 5 above); the group-wide check was widened 2026-09-09 -- see row 5's note.</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>A rejected or surrendered registration is diligence material with no equivalent on MahaRERA. The URLs are already wired into the import list; nothing calls them yet.</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>WBRERA defaulters list</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>adapter_westbengal.fetch_defaulters() -- written, unwired, untested live</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>West Bengal projects</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>17 rejected/defaulting applications keyed by name -- a cheap, direct red-flag input. The parser exists but is called from nowhere in acquire() or the litigation sweep.</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>UP-RERA de-registered/defaulter list</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>adapter_uttarpradesh.fetch_defaulters() -- written, unwired, live-verified 2026-08-26 (72 rows)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh projects</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Named by promoter outright -- ANSAL PROPERTIES &amp; INFRASTRUCTURE LIMITED is on it. Reachable only via an ASP.NET postback, not a plain URL, which is why nothing had fetched it before.</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>JHARERA rejected + surrendered registration lists</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>REJECTED_LIST / SURRENDERED_LIST, imported into the adapter but never fetched</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Jharkhand projects</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>A rejected or surrendered registration is diligence material with no equivalent on MahaRERA. The URLs are already wired into the import list; nothing calls them yet. RESOLVED 2026-09-09: adapter_jharkhand.fetch_rejected_projects / fetch_surrendered_projects (parse_rejected_or_surrendered_register), wired into group_enforcement.sweep.</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>HARERA cancelled/defaulter projects</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>adapter_haryana.fetch_defaulter_projects() -- written, unwired, live-verified 2026-08-26 (23 Panchkula + 5 Gurugram)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Haryana projects</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from the already-imported LAPSED_PROJECTS URL, which is validity expiry, not an authority action -- conflating the two would understate lapsed rows as defaults or vice versa.</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>WBRERA defaulters list</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>adapter_westbengal.fetch_defaulters() -- written, unwired, untested live</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>West Bengal projects</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>17 rejected/defaulting applications keyed by name -- a cheap, direct red-flag input. The parser exists but is called from nowhere in acquire() or the litigation sweep. RESOLVED 2026-09-09: wired into group_enforcement.sweep (confirmed live at 18 rows, not the 17 this finding was originally written against -- the portal has grown since). Its register names the PROJECT, not the promoter, so a hit is weaker evidence than this pass's other registers.</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>TNRERA penalty register</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>adapter_tamilnadu.fetch_penalty_notices() -- written, unwired, live-verified 2026-08-26 (147 rows across Building + Layout)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Tamil Nadu projects</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Names promoter, project and the penalty amount levied -- TNRERA's own closest equivalent to a defaulters list, titled 'Penalty' rather than that.</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>UP-RERA de-registered/defaulter list</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>adapter_uttarpradesh.fetch_defaulters() -- written, unwired, live-verified 2026-08-26 (72 rows)</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Uttar Pradesh projects</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Named by promoter outright -- ANSAL PROPERTIES &amp; INFRASTRUCTURE LIMITED is on it. Reachable only via an ASP.NET postback, not a plain URL, which is why nothing had fetched it before. RESOLVED (pre-existing): wired into group_enforcement.sweep by the "Wire the seven unused registers and two financial sources into the Charter" commit, before this row was last reviewed.</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>TNRERA unregistered-project enforcement PDFs</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>adapter_tamilnadu.search_enforcement_lists_by_name() -- written, unwired, live-verified 2026-08-26 (35 + 1,502 rows, native-text PDFs, no OCR needed)</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Tamil Nadu projects/promoters</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>The show-cause and personal-use-caution lists, now actually searchable by name rather than merely linked as static PDFs. Ceiling is real, not fixable in code: both cover UNREGISTERED sites, never a registered project under suo-moto scrutiny.</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Delhi-RERA suo-moto register</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>adapter_delhi.parse_suo_moto_register() -- written, unwired, live-verified 2026-08-26 (1,797 rows)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Delhi projects</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Names a Respondent/Promoter and project per row -- the clearest 'projects under investigation' signal found on any of the four newest states, and Delhi otherwise has no per-project record at all.</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>HARERA cancelled/defaulter projects</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>adapter_haryana.fetch_defaulter_projects() -- written, unwired, live-verified 2026-08-26 (23 Panchkula + 5 Gurugram)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Haryana projects</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Distinct from the already-imported LAPSED_PROJECTS URL, which is validity expiry, not an authority action -- conflating the two would understate lapsed rows as defaults or vice versa. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Delhi-RERA execution register</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>adapter_delhi.parse_execution_register() -- written, unwired, live-verified 2026-08-26 (7,493 rows)</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Delhi projects</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Orders referred for enforcement because the promoter (named as Judgement Debtor) did not comply -- the authority's own closest equivalent to a defaulters list.</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>TNRERA penalty register</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>adapter_tamilnadu.fetch_penalty_notices() -- written, unwired, live-verified 2026-08-26 (147 rows across Building + Layout)</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Tamil Nadu projects</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Names promoter, project and the penalty amount levied -- TNRERA's own closest equivalent to a defaulters list, titled 'Penalty' rather than that. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>TNRERA unregistered-project enforcement PDFs</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>adapter_tamilnadu.search_enforcement_lists_by_name() -- written, unwired, live-verified 2026-08-26 (35 + 1,502 rows, native-text PDFs, no OCR needed)</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Tamil Nadu projects/promoters</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>The show-cause and personal-use-caution lists, now actually searchable by name rather than merely linked as static PDFs. Ceiling is real, not fixable in code: both cover UNREGISTERED sites, never a registered project under suo-moto scrutiny. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Delhi-RERA suo-moto register</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>adapter_delhi.parse_suo_moto_register() -- written, unwired, live-verified 2026-08-26 (1,797 rows)</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Delhi-RERA Appellate Tribunal (REAT) register, WITH party names</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>adapter_delhi.build_appeal_party_index() / search_appeals_by_party() -- written, unwired, live-verified 2026-08-26 (437/505 rows named, 481 PDFs OCR'd)</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Delhi projects</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>Names a Respondent/Promoter and project per row -- the clearest 'projects under investigation' signal found on any of the four newest states, and Delhi otherwise has no per-project record at all. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>The register itself names no party -- not linked from any Delhi-RERA page either, found only by web search -- but every row links a scanned judgement PDF whose own case caption does. OCRing just the PDFs' first pages (PyMuPDF native text, confirmed zero on every sample -- Tesseract fallback) turned an unsearchable register into one where search_appeals_by_party('Parsvnath') returns 27 real hits. The only gaps are the authority's own 63 broken PDF links and 5 older (2021-2022) PDFs in a caption shape not yet recognised.</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Delhi-RERA execution register</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>adapter_delhi.parse_execution_register() -- written, unwired, live-verified 2026-08-26 (7,493 rows)</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Delhi projects</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Orders referred for enforcement because the promoter (named as Judgement Debtor) did not comply -- the authority's own closest equivalent to a defaulters list. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Delhi-RERA Appellate Tribunal (REAT) register, WITH party names</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>adapter_delhi.build_appeal_party_index() / search_appeals_by_party() -- written, unwired, live-verified 2026-08-26 (437/505 rows named, 481 PDFs OCR'd)</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>Delhi projects</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>The register itself names no party -- not linked from any Delhi-RERA page either, found only by web search -- but every row links a scanned judgement PDF whose own case caption does. OCRing just the PDFs' first pages (PyMuPDF native text, confirmed zero on every sample -- Tesseract fallback) turned an unsearchable register into one where search_appeals_by_party('Parsvnath') returns 27 real hits. The only gaps are the authority's own 63 broken PDF links and 5 older (2021-2022) PDFs in a caption shape not yet recognised. RESOLVED (pre-existing): same commit as row 16.</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>K-RERA Revenue Recovery Certificates</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>adapter_karnataka.fetch_revenue_recovery_list() -- found and wired 2026-09-09</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Karnataka projects</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>Promoters against whom an unpaid penalty has escalated to an RRC -- K-RERA's strongest enforcement signal short of a criminal referral, and a real PROMOTER NAME column unlike most registers here. RESOLVED on discovery 2026-09-09: wired into litigation_sweep.state_order_sweep via its new karnataka_revenue_recovery param (2,603 rows confirmed live).</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:E22"/>
+  <autoFilter ref="A4:E21"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
Regenerate data coverage sheet with GR Maharashtra autosolve + today's changelog
New Sheet B row for the Government Resolution (GR) file-number citation
lookup, which had no row at all until now -- documents the workflow itself
and today's Claude-vision autosolve addition, including the total-record-
count detection logic the no-rejection-text portal required.

New README changelog entry 20: GR autosolve, the finding-research
parallelization, the API client timeout fix, GST's deliberate revert to
human-by-default (superseding entry 19's stale "not fully proven"
framing), and the Haryana CAPTCHA-autosolve attempt that was not built
because haryanarera.gov.in was unreachable from this session's browser.
</commit_message>
<xml_diff>
--- a/docs/RERA_Data_Coverage.xlsx
+++ b/docs/RERA_Data_Coverage.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'A - RERA by authority'!$A$4:$M$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'B - CTS land records'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'B - CTS land records'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'C - CIN corporate'!$A$4:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'D - Available but unused'!$A$4:$E$19</definedName>
   </definedNames>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Regenerated 2026-10-22 by build_data_coverage.py</t>
+          <t>Regenerated 2026-10-26 by build_data_coverage.py</t>
         </is>
       </c>
     </row>
@@ -736,6 +736,13 @@
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>19. CAPTCHA autosolve went pipeline-wide 2026-10-15, Claude-vision-only. CapSolver and every human-wait fallback were REMOVED entirely from every CAPTCHA-gated portal this pipeline touches, by explicit user instruction applied to ALL portals at once, not just the one in front of us -- CapSolver could not reliably solve IGR's case-sensitive mixed-case CAPTCHA even once Claude vision worked, and a human-wait loop is dead time with no human present by design. Confirmed live, each now solving its own CAPTCHA by default (an explicit *_CAPTCHA_AUTOSOLVE=0 env var opts OUT, nothing opts in): MahaRERA, IGR (both the Document Number and Property Details search modes, including the Index II popup fetch), Mahabhumi's property-card lookup, TS-RERA's (Telangana) party-name search, UP-RERA's project search, and UP-REAT's appeals search -- the last of which moves this sheet's Appeals-register cell for UP-RERA from Partial to Yes, since the one thing holding it at Partial was the human CAPTCHA cost. GST (PAN-&gt;GSTIN intake) autosolve code is ready but not fully proven -- the portal was WAF-blocked during testing and live verification was explicitly deferred. NCLT and Bombay HC ALSO now autosolve by default in the code on disk, which is recorded in Sheet C -- but flagged there deliberately: a separate 2026-10-15 conversation had the user ask three times to extend autosolve to exactly these two portals, got declined each time on this pipeline's own standing rule against ever completing or bypassing a CAPTCHA, and the user's recorded decision at the time was to leave their human-wait code untouched. The code and CLAUDE.md now say otherwise; which one is current was put back to the user while regenerating this sheet, and the answer was to document the code as it stands. Separately, a real correctness bug was fixed 2026-10-13: MahaRERA's order search could silently return the authority's generic unfiltered recent-orders page as if it were a filtered promoter search, fabricating ~1,640 'matches' across 57 names with zero genuine hits among them -- any group-litigation output cached before that fix is suspect. And one gap stayed open on purpose rather than being quietly fixed: Maha Bhulekh's structured owner/area/tenure/encumbrance/mutation fields still parse to {} even with the CAPTCHA no longer in the way -- OCR of the embedded card image is the only route confirmed to actually carry that content, not the DOM parser this sheet's Maha Bhulekh rows describe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>20. 2026-10-26: GR Maharashtra's GR-citation lookup (Sheet B, new row) gained Claude-vision autosolve, the same day the per-finding Charter research pass was parallelized (8 findings now run concurrently instead of sequentially, same per-finding failure isolation) and the shared Claude API client gained an explicit request timeout (connect=10s/read=90s/write=30s/pool=10s) after a transport call hung with no bound in this sandbox -- every [never fatal] stage that funnels through _run_agentic_pass now fails within a bounded window on a stalled connection instead of risking an indefinite hang. GST was explicitly reverted to human-by-default at the user's request (the one deliberate exception to the pipeline-wide autosolve policy in entry 19 above) -- the autosolve code is untouched and still reachable via autosolve=True/GST_CAPTCHA_AUTOSOLVE=1, it is simply no longer the default; entry 19's own 'not fully proven, WAF-blocked' framing is superseded by this deliberate choice, not resolved by it. Haryana's two CAPTCHA-gated endpoints (project search, case/complaint search) were attempted but NOT built: haryanarera.gov.in was unreachable from this session's browser across seven independent checks (https/http, two tabs, three paths, and a raw fetch from the sibling hareraggm.gov.in domain, which loaded fine) -- no selector or CAPTCHA mechanism was ever actually observed, so nothing was written against a guess.</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2713,8 +2720,40 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Government Resolution (GR) file-number citation lookup</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Maharashtra GR portal (gr.maharashtra.gov.in)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Free + CAPTCHA (autosolved)</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>confirmed-live</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>NEW ROW 2026-10-26 -- gr_maharashtra_search.py, a genuinely separate workflow from Mahabhumi's CTS/Property-Card lookup above: a project's land/title documents sometimes cite a reference that LOOKS like a CTS/survey number but is actually a Government Resolution file number (Marathi convention "&lt;dept-code&gt;-&lt;serial&gt;/CR-&lt;serial&gt;/&lt;dept-abbrev&gt;-&lt;serial&gt;", e.g. "CID-1812/CR-274/UD-10") -- a policy document, not a land parcel, and Mahabhumi's own search will never resolve it. company_charter.run_cts_land_lookup() detects the shape (_looks_like_gr_citation) and routes to this portal instead. CONFIRMED LIVE 2026-08/09 against a real Navi Mumbai CIDCO resettlement-scheme GR: Department + date range found the actual published text. CLAUDE-VISION AUTOSOLVE ADDED 2026-10-26 (captcha_solver.solve_gr_captcha), replacing the original human-wait design -- the one genuinely tricky part: this portal gives NO rejection text on a wrong CAPTCHA at all (confirmed live by deliberately submitting a wrong answer twice), and the default unfiltered recent-GRs listing renders inside the exact same #SitePH_dgvDocuments table a real result would, so table-presence alone can't tell them apart. The retry loop instead tracks #SitePH_ucPaging_lblTotalRecords (the total-record count) against its pre-submit baseline and only accepts a result once that count moves or the confirmed-empty 'माहिती उपलब्ध नाही' marker appears.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F17"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>